<commit_message>
Lisää exceliin teksti: Kirjaa käpyväylät yksi tienosa kerrallaan (kukin tienosa omalla rivillään).
</commit_message>
<xml_diff>
--- a/dev-resources/excel/harja_talvihoitoreitit_pohja.xlsx
+++ b/dev-resources/excel/harja_talvihoitoreitit_pohja.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11027"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10531"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/markusva/Downloads/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/markusva/repos/Github/harja/dev-resources/excel/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{21BDED3E-2985-6647-A040-A1A71D87EED2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{F1B24F87-5856-5745-8C8C-E20D69FE2591}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="32980" yWindow="-6320" windowWidth="28800" windowHeight="17500" activeTab="1" xr2:uid="{8084DE53-A81F-1C43-943B-FDF8486ACF4F}"/>
+    <workbookView xWindow="34560" yWindow="-5860" windowWidth="28800" windowHeight="17500" activeTab="1" xr2:uid="{8084DE53-A81F-1C43-943B-FDF8486ACF4F}"/>
   </bookViews>
   <sheets>
     <sheet name="Reittien nimet &amp; kalusto" sheetId="3" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="35">
   <si>
     <t>HARJA Talvihoitoreitit</t>
   </si>
@@ -141,12 +141,15 @@
   <si>
     <t>Pituus (km)*</t>
   </si>
+  <si>
+    <t>Kirjaa käpyväylät yksi tienosa kerrallaan (kukin tienosa omalla rivillään).</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -179,6 +182,12 @@
       <color theme="1"/>
       <name val="Aptos Narrow"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="6">
@@ -287,7 +296,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -328,6 +337,7 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normaali" xfId="0" builtinId="0"/>
@@ -3511,7 +3521,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0389D453-6774-C346-BDCD-6729BBE93D77}">
-  <dimension ref="A1:K499"/>
+  <dimension ref="A1:K500"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="20.83203125" style="1" customWidth="1"/>
@@ -3537,53 +3547,51 @@
         <v>23</v>
       </c>
     </row>
-    <row r="4" spans="1:11" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="7" t="s">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A4" s="24" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A5" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="B4" s="8"/>
-      <c r="C4" s="8"/>
-      <c r="D4" s="8"/>
-      <c r="E4" s="8"/>
-      <c r="F4" s="8"/>
-      <c r="G4" s="8"/>
-      <c r="H4" s="21"/>
-      <c r="I4" s="7"/>
-      <c r="J4" s="7"/>
-      <c r="K4" s="7"/>
-    </row>
-    <row r="5" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="5" t="s">
+      <c r="B5" s="8"/>
+      <c r="C5" s="8"/>
+      <c r="D5" s="8"/>
+      <c r="E5" s="8"/>
+      <c r="F5" s="8"/>
+      <c r="G5" s="8"/>
+      <c r="H5" s="21"/>
+      <c r="I5" s="7"/>
+      <c r="J5" s="7"/>
+      <c r="K5" s="7"/>
+    </row>
+    <row r="6" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A6" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="6" t="s">
+      <c r="B6" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="C5" s="6" t="s">
+      <c r="C6" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="D5" s="6" t="s">
+      <c r="D6" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="E5" s="6" t="s">
+      <c r="E6" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="F5" s="6" t="s">
+      <c r="F6" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="G5" s="6" t="s">
+      <c r="G6" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="H5" s="22" t="s">
+      <c r="H6" s="22" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="B6" s="11"/>
-      <c r="C6" s="11"/>
-      <c r="D6" s="11"/>
-      <c r="E6" s="11"/>
-      <c r="F6" s="11"/>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.2">
       <c r="B7" s="11"/>
@@ -3650,16 +3658,16 @@
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.2">
       <c r="B16" s="11"/>
-      <c r="C16" s="11" t="s">
-        <v>13</v>
-      </c>
+      <c r="C16" s="11"/>
       <c r="D16" s="11"/>
       <c r="E16" s="11"/>
       <c r="F16" s="11"/>
     </row>
     <row r="17" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B17" s="11"/>
-      <c r="C17" s="11"/>
+      <c r="C17" s="11" t="s">
+        <v>13</v>
+      </c>
       <c r="D17" s="11"/>
       <c r="E17" s="11"/>
       <c r="F17" s="11"/>
@@ -7037,6 +7045,13 @@
       <c r="D499" s="11"/>
       <c r="E499" s="11"/>
       <c r="F499" s="11"/>
+    </row>
+    <row r="500" spans="2:6" x14ac:dyDescent="0.2">
+      <c r="B500" s="11"/>
+      <c r="C500" s="11"/>
+      <c r="D500" s="11"/>
+      <c r="E500" s="11"/>
+      <c r="F500" s="11"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -7047,13 +7062,13 @@
           <x14:formula1>
             <xm:f>Valinnat!$B$2:$B$13</xm:f>
           </x14:formula1>
-          <xm:sqref>G6:G1048576</xm:sqref>
+          <xm:sqref>G7:G1048576</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{678C7DB7-CB21-0F43-984F-23641463B6AF}">
           <x14:formula1>
             <xm:f>'Reittien nimet &amp; kalusto'!$A$5:$A$1630</xm:f>
           </x14:formula1>
-          <xm:sqref>A6:A1048576</xm:sqref>
+          <xm:sqref>A7:A1048576</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>

</xml_diff>